<commit_message>
datos: actualización automática 2026-10-06
CEPOES-Producer-Workflow: .github/workflows/actualizar.yml
CEPOES-Producer-Run: 37504203498
CEPOES-Producer-Attempt: 1
CEPOES-Producer-Input: 828dd7390ab6385d205960aed90d416bbedcb36d
</commit_message>
<xml_diff>
--- a/idecba/industria_ing.xlsx
+++ b/idecba/industria_ing.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\SRV03\Centro_Doc\BANCO DE DATOS\CARPETAS BCO DE DATOS\INDUSTRIA\INGRESOS FABRILES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\srv03\Centro_Doc\BANCO DE DATOS\CARPETAS BCO DE DATOS\INDUSTRIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25455" windowHeight="8745"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11730"/>
   </bookViews>
   <sheets>
     <sheet name="ee_industria_ingresos_fabriles" sheetId="2" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="63">
   <si>
     <t xml:space="preserve">Alimentos, bebidas y tabaco </t>
   </si>
@@ -224,10 +224,10 @@
     <t>2025*</t>
   </si>
   <si>
-    <t>Ingresos fabriles por rama de actividad en valores corrientes y constantes (Índice base octubre 2001 = 100). Ciudad de Buenos Aires. Octubre 2001/Marzo 2026</t>
+    <t>2026*</t>
   </si>
   <si>
-    <t>2026*</t>
+    <t>Ingresos fabriles por rama de actividad en valores corrientes y constantes (Índice base octubre 2001 = 100). Ciudad de Buenos Aires. Octubre 2001/Junio 2026</t>
   </si>
 </sst>
 </file>
@@ -555,7 +555,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="51">
+  <borders count="52">
     <border>
       <left/>
       <right/>
@@ -1161,6 +1161,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1446,7 +1457,7 @@
       <alignment horizontal="right" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1455,11 +1466,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1469,18 +1486,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="3" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="3" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1500,13 +1505,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="3" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="3" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="43" xfId="35" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1866,7 +1877,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:V475"/>
+  <dimension ref="A1:V478"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.28515625" style="15" customWidth="1"/>
@@ -1877,20 +1888,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="92" t="s">
-        <v>61</v>
-      </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="92"/>
-      <c r="H1" s="92"/>
-      <c r="I1" s="92"/>
-      <c r="J1" s="92"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
+      <c r="A1" s="101" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="101"/>
+      <c r="G1" s="101"/>
+      <c r="H1" s="101"/>
+      <c r="I1" s="101"/>
+      <c r="J1" s="101"/>
+      <c r="K1" s="101"/>
+      <c r="L1" s="101"/>
       <c r="M1" s="5"/>
       <c r="N1" s="5"/>
       <c r="O1" s="4"/>
@@ -1903,40 +1914,40 @@
       <c r="V1" s="4"/>
     </row>
     <row r="2" spans="1:22" s="4" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="99" t="s">
+      <c r="A2" s="97" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="100" t="s">
+      <c r="B2" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="93" t="s">
+      <c r="C2" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="96" t="s">
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
+      <c r="L2" s="104"/>
+      <c r="M2" s="94" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="97"/>
-      <c r="O2" s="97"/>
-      <c r="P2" s="97"/>
-      <c r="Q2" s="97"/>
-      <c r="R2" s="97"/>
-      <c r="S2" s="97"/>
-      <c r="T2" s="97"/>
-      <c r="U2" s="97"/>
-      <c r="V2" s="98"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="95"/>
+      <c r="Q2" s="95"/>
+      <c r="R2" s="95"/>
+      <c r="S2" s="95"/>
+      <c r="T2" s="95"/>
+      <c r="U2" s="95"/>
+      <c r="V2" s="96"/>
     </row>
     <row r="3" spans="1:22" ht="66" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="91"/>
-      <c r="B3" s="101"/>
+      <c r="A3" s="93"/>
+      <c r="B3" s="99"/>
       <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
@@ -1999,7 +2010,7 @@
       </c>
     </row>
     <row r="4" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="89">
+      <c r="A4" s="91">
         <v>2001</v>
       </c>
       <c r="B4" s="16" t="s">
@@ -2067,7 +2078,7 @@
       </c>
     </row>
     <row r="5" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="90"/>
+      <c r="A5" s="92"/>
       <c r="B5" s="17" t="s">
         <v>14</v>
       </c>
@@ -2133,7 +2144,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="91"/>
+      <c r="A6" s="93"/>
       <c r="B6" s="18" t="s">
         <v>15</v>
       </c>
@@ -2199,7 +2210,7 @@
       </c>
     </row>
     <row r="7" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="90">
+      <c r="A7" s="92">
         <v>2002</v>
       </c>
       <c r="B7" s="17" t="s">
@@ -2267,7 +2278,7 @@
       </c>
     </row>
     <row r="8" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="90"/>
+      <c r="A8" s="92"/>
       <c r="B8" s="17" t="s">
         <v>17</v>
       </c>
@@ -2333,7 +2344,7 @@
       </c>
     </row>
     <row r="9" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="90"/>
+      <c r="A9" s="92"/>
       <c r="B9" s="17" t="s">
         <v>18</v>
       </c>
@@ -2399,7 +2410,7 @@
       </c>
     </row>
     <row r="10" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="90"/>
+      <c r="A10" s="92"/>
       <c r="B10" s="17" t="s">
         <v>19</v>
       </c>
@@ -2465,7 +2476,7 @@
       </c>
     </row>
     <row r="11" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="90"/>
+      <c r="A11" s="92"/>
       <c r="B11" s="17" t="s">
         <v>20</v>
       </c>
@@ -2531,7 +2542,7 @@
       </c>
     </row>
     <row r="12" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="90"/>
+      <c r="A12" s="92"/>
       <c r="B12" s="17" t="s">
         <v>21</v>
       </c>
@@ -2597,7 +2608,7 @@
       </c>
     </row>
     <row r="13" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="90"/>
+      <c r="A13" s="92"/>
       <c r="B13" s="17" t="s">
         <v>22</v>
       </c>
@@ -2663,7 +2674,7 @@
       </c>
     </row>
     <row r="14" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="90"/>
+      <c r="A14" s="92"/>
       <c r="B14" s="17" t="s">
         <v>23</v>
       </c>
@@ -2729,7 +2740,7 @@
       </c>
     </row>
     <row r="15" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="90"/>
+      <c r="A15" s="92"/>
       <c r="B15" s="17" t="s">
         <v>24</v>
       </c>
@@ -2795,7 +2806,7 @@
       </c>
     </row>
     <row r="16" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="90"/>
+      <c r="A16" s="92"/>
       <c r="B16" s="17" t="s">
         <v>13</v>
       </c>
@@ -2861,7 +2872,7 @@
       </c>
     </row>
     <row r="17" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="90"/>
+      <c r="A17" s="92"/>
       <c r="B17" s="17" t="s">
         <v>14</v>
       </c>
@@ -2927,7 +2938,7 @@
       </c>
     </row>
     <row r="18" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="91"/>
+      <c r="A18" s="93"/>
       <c r="B18" s="18" t="s">
         <v>15</v>
       </c>
@@ -2993,7 +3004,7 @@
       </c>
     </row>
     <row r="19" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="90">
+      <c r="A19" s="92">
         <v>2003</v>
       </c>
       <c r="B19" s="17" t="s">
@@ -3061,7 +3072,7 @@
       </c>
     </row>
     <row r="20" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="90"/>
+      <c r="A20" s="92"/>
       <c r="B20" s="17" t="s">
         <v>17</v>
       </c>
@@ -3127,7 +3138,7 @@
       </c>
     </row>
     <row r="21" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="90"/>
+      <c r="A21" s="92"/>
       <c r="B21" s="17" t="s">
         <v>18</v>
       </c>
@@ -3193,7 +3204,7 @@
       </c>
     </row>
     <row r="22" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="90"/>
+      <c r="A22" s="92"/>
       <c r="B22" s="17" t="s">
         <v>19</v>
       </c>
@@ -3259,7 +3270,7 @@
       </c>
     </row>
     <row r="23" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="90"/>
+      <c r="A23" s="92"/>
       <c r="B23" s="17" t="s">
         <v>20</v>
       </c>
@@ -3325,7 +3336,7 @@
       </c>
     </row>
     <row r="24" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="90"/>
+      <c r="A24" s="92"/>
       <c r="B24" s="17" t="s">
         <v>21</v>
       </c>
@@ -3391,7 +3402,7 @@
       </c>
     </row>
     <row r="25" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="90"/>
+      <c r="A25" s="92"/>
       <c r="B25" s="17" t="s">
         <v>22</v>
       </c>
@@ -3457,7 +3468,7 @@
       </c>
     </row>
     <row r="26" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="90"/>
+      <c r="A26" s="92"/>
       <c r="B26" s="17" t="s">
         <v>23</v>
       </c>
@@ -3523,7 +3534,7 @@
       </c>
     </row>
     <row r="27" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="90"/>
+      <c r="A27" s="92"/>
       <c r="B27" s="17" t="s">
         <v>24</v>
       </c>
@@ -3589,7 +3600,7 @@
       </c>
     </row>
     <row r="28" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="90"/>
+      <c r="A28" s="92"/>
       <c r="B28" s="17" t="s">
         <v>13</v>
       </c>
@@ -3655,7 +3666,7 @@
       </c>
     </row>
     <row r="29" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="90"/>
+      <c r="A29" s="92"/>
       <c r="B29" s="17" t="s">
         <v>14</v>
       </c>
@@ -3721,7 +3732,7 @@
       </c>
     </row>
     <row r="30" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="91"/>
+      <c r="A30" s="93"/>
       <c r="B30" s="18" t="s">
         <v>15</v>
       </c>
@@ -3787,7 +3798,7 @@
       </c>
     </row>
     <row r="31" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="90">
+      <c r="A31" s="92">
         <v>2004</v>
       </c>
       <c r="B31" s="17" t="s">
@@ -3855,7 +3866,7 @@
       </c>
     </row>
     <row r="32" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="90"/>
+      <c r="A32" s="92"/>
       <c r="B32" s="17" t="s">
         <v>17</v>
       </c>
@@ -3921,7 +3932,7 @@
       </c>
     </row>
     <row r="33" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="90"/>
+      <c r="A33" s="92"/>
       <c r="B33" s="17" t="s">
         <v>18</v>
       </c>
@@ -3987,7 +3998,7 @@
       </c>
     </row>
     <row r="34" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="90"/>
+      <c r="A34" s="92"/>
       <c r="B34" s="17" t="s">
         <v>19</v>
       </c>
@@ -4053,7 +4064,7 @@
       </c>
     </row>
     <row r="35" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="90"/>
+      <c r="A35" s="92"/>
       <c r="B35" s="17" t="s">
         <v>20</v>
       </c>
@@ -4119,7 +4130,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="90"/>
+      <c r="A36" s="92"/>
       <c r="B36" s="17" t="s">
         <v>21</v>
       </c>
@@ -4185,7 +4196,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="90"/>
+      <c r="A37" s="92"/>
       <c r="B37" s="17" t="s">
         <v>22</v>
       </c>
@@ -4251,7 +4262,7 @@
       </c>
     </row>
     <row r="38" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="90"/>
+      <c r="A38" s="92"/>
       <c r="B38" s="17" t="s">
         <v>23</v>
       </c>
@@ -4317,7 +4328,7 @@
       </c>
     </row>
     <row r="39" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="90"/>
+      <c r="A39" s="92"/>
       <c r="B39" s="17" t="s">
         <v>24</v>
       </c>
@@ -4383,7 +4394,7 @@
       </c>
     </row>
     <row r="40" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="90"/>
+      <c r="A40" s="92"/>
       <c r="B40" s="17" t="s">
         <v>13</v>
       </c>
@@ -4449,7 +4460,7 @@
       </c>
     </row>
     <row r="41" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="90"/>
+      <c r="A41" s="92"/>
       <c r="B41" s="17" t="s">
         <v>14</v>
       </c>
@@ -4515,7 +4526,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="91"/>
+      <c r="A42" s="93"/>
       <c r="B42" s="18" t="s">
         <v>15</v>
       </c>
@@ -4581,7 +4592,7 @@
       </c>
     </row>
     <row r="43" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="90">
+      <c r="A43" s="92">
         <v>2005</v>
       </c>
       <c r="B43" s="17" t="s">
@@ -4649,7 +4660,7 @@
       </c>
     </row>
     <row r="44" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="90"/>
+      <c r="A44" s="92"/>
       <c r="B44" s="17" t="s">
         <v>17</v>
       </c>
@@ -4715,7 +4726,7 @@
       </c>
     </row>
     <row r="45" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="90"/>
+      <c r="A45" s="92"/>
       <c r="B45" s="17" t="s">
         <v>18</v>
       </c>
@@ -4781,7 +4792,7 @@
       </c>
     </row>
     <row r="46" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="90"/>
+      <c r="A46" s="92"/>
       <c r="B46" s="17" t="s">
         <v>19</v>
       </c>
@@ -4847,7 +4858,7 @@
       </c>
     </row>
     <row r="47" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="90"/>
+      <c r="A47" s="92"/>
       <c r="B47" s="17" t="s">
         <v>20</v>
       </c>
@@ -4913,7 +4924,7 @@
       </c>
     </row>
     <row r="48" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="90"/>
+      <c r="A48" s="92"/>
       <c r="B48" s="17" t="s">
         <v>21</v>
       </c>
@@ -4979,7 +4990,7 @@
       </c>
     </row>
     <row r="49" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="90"/>
+      <c r="A49" s="92"/>
       <c r="B49" s="17" t="s">
         <v>22</v>
       </c>
@@ -5045,7 +5056,7 @@
       </c>
     </row>
     <row r="50" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="90"/>
+      <c r="A50" s="92"/>
       <c r="B50" s="17" t="s">
         <v>23</v>
       </c>
@@ -5111,7 +5122,7 @@
       </c>
     </row>
     <row r="51" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="90"/>
+      <c r="A51" s="92"/>
       <c r="B51" s="17" t="s">
         <v>24</v>
       </c>
@@ -5177,7 +5188,7 @@
       </c>
     </row>
     <row r="52" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="90"/>
+      <c r="A52" s="92"/>
       <c r="B52" s="17" t="s">
         <v>13</v>
       </c>
@@ -5243,7 +5254,7 @@
       </c>
     </row>
     <row r="53" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="90"/>
+      <c r="A53" s="92"/>
       <c r="B53" s="17" t="s">
         <v>14</v>
       </c>
@@ -5309,7 +5320,7 @@
       </c>
     </row>
     <row r="54" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="91"/>
+      <c r="A54" s="93"/>
       <c r="B54" s="18" t="s">
         <v>15</v>
       </c>
@@ -5375,7 +5386,7 @@
       </c>
     </row>
     <row r="55" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="90">
+      <c r="A55" s="92">
         <v>2006</v>
       </c>
       <c r="B55" s="17" t="s">
@@ -5443,7 +5454,7 @@
       </c>
     </row>
     <row r="56" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="90"/>
+      <c r="A56" s="92"/>
       <c r="B56" s="17" t="s">
         <v>17</v>
       </c>
@@ -5509,7 +5520,7 @@
       </c>
     </row>
     <row r="57" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="90"/>
+      <c r="A57" s="92"/>
       <c r="B57" s="17" t="s">
         <v>18</v>
       </c>
@@ -5575,7 +5586,7 @@
       </c>
     </row>
     <row r="58" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="90"/>
+      <c r="A58" s="92"/>
       <c r="B58" s="17" t="s">
         <v>19</v>
       </c>
@@ -5641,7 +5652,7 @@
       </c>
     </row>
     <row r="59" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="90"/>
+      <c r="A59" s="92"/>
       <c r="B59" s="17" t="s">
         <v>20</v>
       </c>
@@ -5707,7 +5718,7 @@
       </c>
     </row>
     <row r="60" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="90"/>
+      <c r="A60" s="92"/>
       <c r="B60" s="17" t="s">
         <v>21</v>
       </c>
@@ -5773,7 +5784,7 @@
       </c>
     </row>
     <row r="61" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="90"/>
+      <c r="A61" s="92"/>
       <c r="B61" s="17" t="s">
         <v>22</v>
       </c>
@@ -5839,7 +5850,7 @@
       </c>
     </row>
     <row r="62" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="90"/>
+      <c r="A62" s="92"/>
       <c r="B62" s="17" t="s">
         <v>23</v>
       </c>
@@ -5905,7 +5916,7 @@
       </c>
     </row>
     <row r="63" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="90"/>
+      <c r="A63" s="92"/>
       <c r="B63" s="17" t="s">
         <v>24</v>
       </c>
@@ -5971,7 +5982,7 @@
       </c>
     </row>
     <row r="64" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="90"/>
+      <c r="A64" s="92"/>
       <c r="B64" s="17" t="s">
         <v>13</v>
       </c>
@@ -6037,7 +6048,7 @@
       </c>
     </row>
     <row r="65" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="90"/>
+      <c r="A65" s="92"/>
       <c r="B65" s="17" t="s">
         <v>14</v>
       </c>
@@ -6103,7 +6114,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="91"/>
+      <c r="A66" s="93"/>
       <c r="B66" s="18" t="s">
         <v>15</v>
       </c>
@@ -6169,7 +6180,7 @@
       </c>
     </row>
     <row r="67" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="90">
+      <c r="A67" s="92">
         <v>2007</v>
       </c>
       <c r="B67" s="17" t="s">
@@ -6237,7 +6248,7 @@
       </c>
     </row>
     <row r="68" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="90"/>
+      <c r="A68" s="92"/>
       <c r="B68" s="17" t="s">
         <v>17</v>
       </c>
@@ -6303,7 +6314,7 @@
       </c>
     </row>
     <row r="69" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="90"/>
+      <c r="A69" s="92"/>
       <c r="B69" s="17" t="s">
         <v>18</v>
       </c>
@@ -6369,7 +6380,7 @@
       </c>
     </row>
     <row r="70" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="90"/>
+      <c r="A70" s="92"/>
       <c r="B70" s="17" t="s">
         <v>19</v>
       </c>
@@ -6435,7 +6446,7 @@
       </c>
     </row>
     <row r="71" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="90"/>
+      <c r="A71" s="92"/>
       <c r="B71" s="17" t="s">
         <v>20</v>
       </c>
@@ -6501,7 +6512,7 @@
       </c>
     </row>
     <row r="72" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="90"/>
+      <c r="A72" s="92"/>
       <c r="B72" s="17" t="s">
         <v>21</v>
       </c>
@@ -6567,7 +6578,7 @@
       </c>
     </row>
     <row r="73" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="90"/>
+      <c r="A73" s="92"/>
       <c r="B73" s="17" t="s">
         <v>22</v>
       </c>
@@ -6633,7 +6644,7 @@
       </c>
     </row>
     <row r="74" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="90"/>
+      <c r="A74" s="92"/>
       <c r="B74" s="17" t="s">
         <v>23</v>
       </c>
@@ -6699,7 +6710,7 @@
       </c>
     </row>
     <row r="75" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="90"/>
+      <c r="A75" s="92"/>
       <c r="B75" s="17" t="s">
         <v>24</v>
       </c>
@@ -6765,7 +6776,7 @@
       </c>
     </row>
     <row r="76" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="90"/>
+      <c r="A76" s="92"/>
       <c r="B76" s="17" t="s">
         <v>13</v>
       </c>
@@ -6831,7 +6842,7 @@
       </c>
     </row>
     <row r="77" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="90"/>
+      <c r="A77" s="92"/>
       <c r="B77" s="17" t="s">
         <v>14</v>
       </c>
@@ -6897,7 +6908,7 @@
       </c>
     </row>
     <row r="78" spans="1:22" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="91"/>
+      <c r="A78" s="93"/>
       <c r="B78" s="18" t="s">
         <v>15</v>
       </c>
@@ -6963,7 +6974,7 @@
       </c>
     </row>
     <row r="79" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A79" s="90">
+      <c r="A79" s="92">
         <v>2008</v>
       </c>
       <c r="B79" s="17" t="s">
@@ -7031,7 +7042,7 @@
       </c>
     </row>
     <row r="80" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A80" s="90"/>
+      <c r="A80" s="92"/>
       <c r="B80" s="17" t="s">
         <v>17</v>
       </c>
@@ -7097,7 +7108,7 @@
       </c>
     </row>
     <row r="81" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A81" s="90"/>
+      <c r="A81" s="92"/>
       <c r="B81" s="17" t="s">
         <v>18</v>
       </c>
@@ -7163,7 +7174,7 @@
       </c>
     </row>
     <row r="82" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A82" s="90"/>
+      <c r="A82" s="92"/>
       <c r="B82" s="17" t="s">
         <v>19</v>
       </c>
@@ -7229,7 +7240,7 @@
       </c>
     </row>
     <row r="83" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A83" s="90"/>
+      <c r="A83" s="92"/>
       <c r="B83" s="17" t="s">
         <v>20</v>
       </c>
@@ -7295,7 +7306,7 @@
       </c>
     </row>
     <row r="84" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A84" s="90"/>
+      <c r="A84" s="92"/>
       <c r="B84" s="17" t="s">
         <v>21</v>
       </c>
@@ -7361,7 +7372,7 @@
       </c>
     </row>
     <row r="85" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A85" s="90"/>
+      <c r="A85" s="92"/>
       <c r="B85" s="17" t="s">
         <v>22</v>
       </c>
@@ -7427,7 +7438,7 @@
       </c>
     </row>
     <row r="86" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A86" s="90"/>
+      <c r="A86" s="92"/>
       <c r="B86" s="17" t="s">
         <v>23</v>
       </c>
@@ -7493,7 +7504,7 @@
       </c>
     </row>
     <row r="87" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A87" s="90"/>
+      <c r="A87" s="92"/>
       <c r="B87" s="17" t="s">
         <v>24</v>
       </c>
@@ -7559,7 +7570,7 @@
       </c>
     </row>
     <row r="88" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A88" s="90"/>
+      <c r="A88" s="92"/>
       <c r="B88" s="17" t="s">
         <v>13</v>
       </c>
@@ -7625,7 +7636,7 @@
       </c>
     </row>
     <row r="89" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A89" s="90"/>
+      <c r="A89" s="92"/>
       <c r="B89" s="17" t="s">
         <v>14</v>
       </c>
@@ -7691,7 +7702,7 @@
       </c>
     </row>
     <row r="90" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A90" s="91"/>
+      <c r="A90" s="93"/>
       <c r="B90" s="18" t="s">
         <v>15</v>
       </c>
@@ -7757,7 +7768,7 @@
       </c>
     </row>
     <row r="91" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A91" s="89">
+      <c r="A91" s="91">
         <v>2009</v>
       </c>
       <c r="B91" s="17" t="s">
@@ -7825,7 +7836,7 @@
       </c>
     </row>
     <row r="92" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A92" s="90"/>
+      <c r="A92" s="92"/>
       <c r="B92" s="17" t="s">
         <v>17</v>
       </c>
@@ -7891,7 +7902,7 @@
       </c>
     </row>
     <row r="93" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A93" s="90"/>
+      <c r="A93" s="92"/>
       <c r="B93" s="17" t="s">
         <v>18</v>
       </c>
@@ -7957,7 +7968,7 @@
       </c>
     </row>
     <row r="94" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A94" s="90"/>
+      <c r="A94" s="92"/>
       <c r="B94" s="17" t="s">
         <v>19</v>
       </c>
@@ -8023,7 +8034,7 @@
       </c>
     </row>
     <row r="95" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A95" s="90"/>
+      <c r="A95" s="92"/>
       <c r="B95" s="17" t="s">
         <v>20</v>
       </c>
@@ -8089,7 +8100,7 @@
       </c>
     </row>
     <row r="96" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A96" s="90"/>
+      <c r="A96" s="92"/>
       <c r="B96" s="17" t="s">
         <v>21</v>
       </c>
@@ -8155,7 +8166,7 @@
       </c>
     </row>
     <row r="97" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A97" s="90"/>
+      <c r="A97" s="92"/>
       <c r="B97" s="17" t="s">
         <v>22</v>
       </c>
@@ -8221,7 +8232,7 @@
       </c>
     </row>
     <row r="98" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A98" s="90"/>
+      <c r="A98" s="92"/>
       <c r="B98" s="17" t="s">
         <v>23</v>
       </c>
@@ -8287,7 +8298,7 @@
       </c>
     </row>
     <row r="99" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A99" s="90"/>
+      <c r="A99" s="92"/>
       <c r="B99" s="17" t="s">
         <v>24</v>
       </c>
@@ -8353,7 +8364,7 @@
       </c>
     </row>
     <row r="100" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A100" s="90"/>
+      <c r="A100" s="92"/>
       <c r="B100" s="17" t="s">
         <v>13</v>
       </c>
@@ -8419,7 +8430,7 @@
       </c>
     </row>
     <row r="101" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A101" s="90"/>
+      <c r="A101" s="92"/>
       <c r="B101" s="17" t="s">
         <v>14</v>
       </c>
@@ -8485,7 +8496,7 @@
       </c>
     </row>
     <row r="102" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A102" s="91"/>
+      <c r="A102" s="93"/>
       <c r="B102" s="18" t="s">
         <v>15</v>
       </c>
@@ -8551,7 +8562,7 @@
       </c>
     </row>
     <row r="103" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A103" s="89">
+      <c r="A103" s="91">
         <v>2010</v>
       </c>
       <c r="B103" s="17" t="s">
@@ -8619,7 +8630,7 @@
       </c>
     </row>
     <row r="104" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A104" s="90"/>
+      <c r="A104" s="92"/>
       <c r="B104" s="17" t="s">
         <v>17</v>
       </c>
@@ -8685,7 +8696,7 @@
       </c>
     </row>
     <row r="105" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A105" s="90"/>
+      <c r="A105" s="92"/>
       <c r="B105" s="17" t="s">
         <v>18</v>
       </c>
@@ -8751,7 +8762,7 @@
       </c>
     </row>
     <row r="106" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A106" s="90"/>
+      <c r="A106" s="92"/>
       <c r="B106" s="17" t="s">
         <v>19</v>
       </c>
@@ -8817,7 +8828,7 @@
       </c>
     </row>
     <row r="107" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A107" s="90"/>
+      <c r="A107" s="92"/>
       <c r="B107" s="17" t="s">
         <v>20</v>
       </c>
@@ -8883,7 +8894,7 @@
       </c>
     </row>
     <row r="108" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A108" s="90"/>
+      <c r="A108" s="92"/>
       <c r="B108" s="17" t="s">
         <v>21</v>
       </c>
@@ -8949,7 +8960,7 @@
       </c>
     </row>
     <row r="109" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A109" s="90"/>
+      <c r="A109" s="92"/>
       <c r="B109" s="17" t="s">
         <v>22</v>
       </c>
@@ -9015,7 +9026,7 @@
       </c>
     </row>
     <row r="110" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A110" s="90"/>
+      <c r="A110" s="92"/>
       <c r="B110" s="17" t="s">
         <v>23</v>
       </c>
@@ -9081,7 +9092,7 @@
       </c>
     </row>
     <row r="111" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A111" s="90"/>
+      <c r="A111" s="92"/>
       <c r="B111" s="17" t="s">
         <v>24</v>
       </c>
@@ -9147,7 +9158,7 @@
       </c>
     </row>
     <row r="112" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A112" s="90"/>
+      <c r="A112" s="92"/>
       <c r="B112" s="17" t="s">
         <v>13</v>
       </c>
@@ -9213,7 +9224,7 @@
       </c>
     </row>
     <row r="113" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A113" s="90"/>
+      <c r="A113" s="92"/>
       <c r="B113" s="17" t="s">
         <v>14</v>
       </c>
@@ -9279,7 +9290,7 @@
       </c>
     </row>
     <row r="114" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A114" s="91"/>
+      <c r="A114" s="93"/>
       <c r="B114" s="18" t="s">
         <v>15</v>
       </c>
@@ -9345,7 +9356,7 @@
       </c>
     </row>
     <row r="115" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A115" s="89">
+      <c r="A115" s="91">
         <v>2011</v>
       </c>
       <c r="B115" s="17" t="s">
@@ -9413,7 +9424,7 @@
       </c>
     </row>
     <row r="116" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A116" s="90"/>
+      <c r="A116" s="92"/>
       <c r="B116" s="17" t="s">
         <v>17</v>
       </c>
@@ -9479,7 +9490,7 @@
       </c>
     </row>
     <row r="117" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A117" s="90"/>
+      <c r="A117" s="92"/>
       <c r="B117" s="17" t="s">
         <v>18</v>
       </c>
@@ -9545,7 +9556,7 @@
       </c>
     </row>
     <row r="118" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A118" s="90"/>
+      <c r="A118" s="92"/>
       <c r="B118" s="17" t="s">
         <v>19</v>
       </c>
@@ -9611,7 +9622,7 @@
       </c>
     </row>
     <row r="119" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A119" s="90"/>
+      <c r="A119" s="92"/>
       <c r="B119" s="17" t="s">
         <v>20</v>
       </c>
@@ -9677,7 +9688,7 @@
       </c>
     </row>
     <row r="120" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A120" s="90"/>
+      <c r="A120" s="92"/>
       <c r="B120" s="17" t="s">
         <v>21</v>
       </c>
@@ -9743,7 +9754,7 @@
       </c>
     </row>
     <row r="121" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A121" s="90"/>
+      <c r="A121" s="92"/>
       <c r="B121" s="17" t="s">
         <v>22</v>
       </c>
@@ -9809,7 +9820,7 @@
       </c>
     </row>
     <row r="122" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A122" s="90"/>
+      <c r="A122" s="92"/>
       <c r="B122" s="17" t="s">
         <v>23</v>
       </c>
@@ -9875,7 +9886,7 @@
       </c>
     </row>
     <row r="123" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A123" s="90"/>
+      <c r="A123" s="92"/>
       <c r="B123" s="17" t="s">
         <v>24</v>
       </c>
@@ -9941,7 +9952,7 @@
       </c>
     </row>
     <row r="124" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A124" s="90"/>
+      <c r="A124" s="92"/>
       <c r="B124" s="17" t="s">
         <v>13</v>
       </c>
@@ -10007,7 +10018,7 @@
       </c>
     </row>
     <row r="125" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A125" s="90"/>
+      <c r="A125" s="92"/>
       <c r="B125" s="17" t="s">
         <v>14</v>
       </c>
@@ -10073,7 +10084,7 @@
       </c>
     </row>
     <row r="126" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A126" s="91"/>
+      <c r="A126" s="93"/>
       <c r="B126" s="18" t="s">
         <v>15</v>
       </c>
@@ -10139,7 +10150,7 @@
       </c>
     </row>
     <row r="127" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A127" s="89">
+      <c r="A127" s="91">
         <v>2012</v>
       </c>
       <c r="B127" s="17" t="s">
@@ -10207,7 +10218,7 @@
       </c>
     </row>
     <row r="128" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A128" s="90"/>
+      <c r="A128" s="92"/>
       <c r="B128" s="17" t="s">
         <v>17</v>
       </c>
@@ -10273,7 +10284,7 @@
       </c>
     </row>
     <row r="129" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A129" s="90"/>
+      <c r="A129" s="92"/>
       <c r="B129" s="17" t="s">
         <v>18</v>
       </c>
@@ -10339,7 +10350,7 @@
       </c>
     </row>
     <row r="130" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A130" s="90"/>
+      <c r="A130" s="92"/>
       <c r="B130" s="17" t="s">
         <v>19</v>
       </c>
@@ -10405,7 +10416,7 @@
       </c>
     </row>
     <row r="131" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A131" s="90"/>
+      <c r="A131" s="92"/>
       <c r="B131" s="17" t="s">
         <v>20</v>
       </c>
@@ -10471,7 +10482,7 @@
       </c>
     </row>
     <row r="132" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A132" s="90"/>
+      <c r="A132" s="92"/>
       <c r="B132" s="17" t="s">
         <v>21</v>
       </c>
@@ -10537,7 +10548,7 @@
       </c>
     </row>
     <row r="133" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A133" s="90"/>
+      <c r="A133" s="92"/>
       <c r="B133" s="17" t="s">
         <v>22</v>
       </c>
@@ -10603,7 +10614,7 @@
       </c>
     </row>
     <row r="134" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A134" s="90"/>
+      <c r="A134" s="92"/>
       <c r="B134" s="17" t="s">
         <v>23</v>
       </c>
@@ -10669,7 +10680,7 @@
       </c>
     </row>
     <row r="135" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A135" s="90"/>
+      <c r="A135" s="92"/>
       <c r="B135" s="17" t="s">
         <v>24</v>
       </c>
@@ -10735,7 +10746,7 @@
       </c>
     </row>
     <row r="136" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A136" s="90"/>
+      <c r="A136" s="92"/>
       <c r="B136" s="17" t="s">
         <v>13</v>
       </c>
@@ -10801,7 +10812,7 @@
       </c>
     </row>
     <row r="137" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A137" s="90"/>
+      <c r="A137" s="92"/>
       <c r="B137" s="17" t="s">
         <v>14</v>
       </c>
@@ -10867,7 +10878,7 @@
       </c>
     </row>
     <row r="138" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A138" s="91"/>
+      <c r="A138" s="93"/>
       <c r="B138" s="18" t="s">
         <v>15</v>
       </c>
@@ -10933,7 +10944,7 @@
       </c>
     </row>
     <row r="139" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A139" s="89">
+      <c r="A139" s="91">
         <v>2013</v>
       </c>
       <c r="B139" s="16" t="s">
@@ -11001,7 +11012,7 @@
       </c>
     </row>
     <row r="140" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A140" s="90"/>
+      <c r="A140" s="92"/>
       <c r="B140" s="17" t="s">
         <v>17</v>
       </c>
@@ -11067,7 +11078,7 @@
       </c>
     </row>
     <row r="141" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A141" s="90"/>
+      <c r="A141" s="92"/>
       <c r="B141" s="17" t="s">
         <v>18</v>
       </c>
@@ -11133,7 +11144,7 @@
       </c>
     </row>
     <row r="142" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A142" s="90"/>
+      <c r="A142" s="92"/>
       <c r="B142" s="17" t="s">
         <v>19</v>
       </c>
@@ -11199,7 +11210,7 @@
       </c>
     </row>
     <row r="143" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A143" s="90"/>
+      <c r="A143" s="92"/>
       <c r="B143" s="17" t="s">
         <v>20</v>
       </c>
@@ -11265,7 +11276,7 @@
       </c>
     </row>
     <row r="144" spans="1:22" s="12" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A144" s="90"/>
+      <c r="A144" s="92"/>
       <c r="B144" s="43" t="s">
         <v>21</v>
       </c>
@@ -11331,7 +11342,7 @@
       </c>
     </row>
     <row r="145" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="90"/>
+      <c r="A145" s="92"/>
       <c r="B145" s="17" t="s">
         <v>22</v>
       </c>
@@ -11397,7 +11408,7 @@
       </c>
     </row>
     <row r="146" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="90"/>
+      <c r="A146" s="92"/>
       <c r="B146" s="43" t="s">
         <v>23</v>
       </c>
@@ -11463,7 +11474,7 @@
       </c>
     </row>
     <row r="147" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="90"/>
+      <c r="A147" s="92"/>
       <c r="B147" s="44" t="s">
         <v>26</v>
       </c>
@@ -11529,7 +11540,7 @@
       </c>
     </row>
     <row r="148" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="90"/>
+      <c r="A148" s="92"/>
       <c r="B148" s="44" t="s">
         <v>13</v>
       </c>
@@ -11595,7 +11606,7 @@
       </c>
     </row>
     <row r="149" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A149" s="90"/>
+      <c r="A149" s="92"/>
       <c r="B149" s="44" t="s">
         <v>14</v>
       </c>
@@ -11661,7 +11672,7 @@
       </c>
     </row>
     <row r="150" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A150" s="91"/>
+      <c r="A150" s="93"/>
       <c r="B150" s="46" t="s">
         <v>15</v>
       </c>
@@ -11727,7 +11738,7 @@
       </c>
     </row>
     <row r="151" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="89">
+      <c r="A151" s="91">
         <v>2014</v>
       </c>
       <c r="B151" s="16" t="s">
@@ -11795,7 +11806,7 @@
       </c>
     </row>
     <row r="152" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="90"/>
+      <c r="A152" s="92"/>
       <c r="B152" s="17" t="s">
         <v>17</v>
       </c>
@@ -11861,7 +11872,7 @@
       </c>
     </row>
     <row r="153" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="90"/>
+      <c r="A153" s="92"/>
       <c r="B153" s="43" t="s">
         <v>18</v>
       </c>
@@ -11927,7 +11938,7 @@
       </c>
     </row>
     <row r="154" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="90"/>
+      <c r="A154" s="92"/>
       <c r="B154" s="43" t="s">
         <v>19</v>
       </c>
@@ -11993,7 +12004,7 @@
       </c>
     </row>
     <row r="155" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="90"/>
+      <c r="A155" s="92"/>
       <c r="B155" s="43" t="s">
         <v>20</v>
       </c>
@@ -12059,7 +12070,7 @@
       </c>
     </row>
     <row r="156" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A156" s="90"/>
+      <c r="A156" s="92"/>
       <c r="B156" s="43" t="s">
         <v>21</v>
       </c>
@@ -12125,7 +12136,7 @@
       </c>
     </row>
     <row r="157" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A157" s="90"/>
+      <c r="A157" s="92"/>
       <c r="B157" s="17" t="s">
         <v>22</v>
       </c>
@@ -12191,7 +12202,7 @@
       </c>
     </row>
     <row r="158" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A158" s="90"/>
+      <c r="A158" s="92"/>
       <c r="B158" s="43" t="s">
         <v>23</v>
       </c>
@@ -12257,7 +12268,7 @@
       </c>
     </row>
     <row r="159" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="90"/>
+      <c r="A159" s="92"/>
       <c r="B159" s="43" t="s">
         <v>26</v>
       </c>
@@ -12323,7 +12334,7 @@
       </c>
     </row>
     <row r="160" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A160" s="90"/>
+      <c r="A160" s="92"/>
       <c r="B160" s="43" t="s">
         <v>13</v>
       </c>
@@ -12389,7 +12400,7 @@
       </c>
     </row>
     <row r="161" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A161" s="90"/>
+      <c r="A161" s="92"/>
       <c r="B161" s="43" t="s">
         <v>14</v>
       </c>
@@ -12455,7 +12466,7 @@
       </c>
     </row>
     <row r="162" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A162" s="91"/>
+      <c r="A162" s="93"/>
       <c r="B162" s="46" t="s">
         <v>15</v>
       </c>
@@ -12521,7 +12532,7 @@
       </c>
     </row>
     <row r="163" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="102">
+      <c r="A163" s="88">
         <v>2015</v>
       </c>
       <c r="B163" s="16" t="s">
@@ -12589,7 +12600,7 @@
       </c>
     </row>
     <row r="164" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="103"/>
+      <c r="A164" s="89"/>
       <c r="B164" s="17" t="s">
         <v>17</v>
       </c>
@@ -12655,7 +12666,7 @@
       </c>
     </row>
     <row r="165" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A165" s="103"/>
+      <c r="A165" s="89"/>
       <c r="B165" s="17" t="s">
         <v>18</v>
       </c>
@@ -12721,7 +12732,7 @@
       </c>
     </row>
     <row r="166" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A166" s="103"/>
+      <c r="A166" s="89"/>
       <c r="B166" s="17" t="s">
         <v>19</v>
       </c>
@@ -12787,7 +12798,7 @@
       </c>
     </row>
     <row r="167" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A167" s="103"/>
+      <c r="A167" s="89"/>
       <c r="B167" s="17" t="s">
         <v>20</v>
       </c>
@@ -12853,7 +12864,7 @@
       </c>
     </row>
     <row r="168" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A168" s="103"/>
+      <c r="A168" s="89"/>
       <c r="B168" s="17" t="s">
         <v>21</v>
       </c>
@@ -12919,7 +12930,7 @@
       </c>
     </row>
     <row r="169" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A169" s="103"/>
+      <c r="A169" s="89"/>
       <c r="B169" s="17" t="s">
         <v>22</v>
       </c>
@@ -12985,7 +12996,7 @@
       </c>
     </row>
     <row r="170" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A170" s="103"/>
+      <c r="A170" s="89"/>
       <c r="B170" s="17" t="s">
         <v>23</v>
       </c>
@@ -13051,7 +13062,7 @@
       </c>
     </row>
     <row r="171" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A171" s="103"/>
+      <c r="A171" s="89"/>
       <c r="B171" s="17" t="s">
         <v>26</v>
       </c>
@@ -13117,7 +13128,7 @@
       </c>
     </row>
     <row r="172" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A172" s="103"/>
+      <c r="A172" s="89"/>
       <c r="B172" s="17" t="s">
         <v>13</v>
       </c>
@@ -13183,7 +13194,7 @@
       </c>
     </row>
     <row r="173" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A173" s="103"/>
+      <c r="A173" s="89"/>
       <c r="B173" s="17" t="s">
         <v>14</v>
       </c>
@@ -13249,7 +13260,7 @@
       </c>
     </row>
     <row r="174" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A174" s="104"/>
+      <c r="A174" s="90"/>
       <c r="B174" s="18" t="s">
         <v>15</v>
       </c>
@@ -18013,7 +18024,7 @@
       </c>
     </row>
     <row r="246" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A246" s="88"/>
+      <c r="A246" s="87"/>
       <c r="B246" s="74" t="s">
         <v>15</v>
       </c>
@@ -18807,7 +18818,7 @@
       </c>
     </row>
     <row r="258" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A258" s="88"/>
+      <c r="A258" s="87"/>
       <c r="B258" s="79" t="s">
         <v>15</v>
       </c>
@@ -19601,7 +19612,7 @@
       </c>
     </row>
     <row r="270" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A270" s="88"/>
+      <c r="A270" s="87"/>
       <c r="B270" s="18" t="s">
         <v>15</v>
       </c>
@@ -20395,7 +20406,7 @@
       </c>
     </row>
     <row r="282" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A282" s="88"/>
+      <c r="A282" s="87"/>
       <c r="B282" s="18" t="s">
         <v>15</v>
       </c>
@@ -21189,7 +21200,7 @@
       </c>
     </row>
     <row r="294" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A294" s="88"/>
+      <c r="A294" s="87"/>
       <c r="B294" s="79" t="s">
         <v>15</v>
       </c>
@@ -21256,7 +21267,7 @@
     </row>
     <row r="295" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A295" s="85" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B295" s="16" t="s">
         <v>16</v>
@@ -21388,145 +21399,274 @@
         <v>125.09382606881042</v>
       </c>
     </row>
-    <row r="297" spans="1:22" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A297" s="87"/>
-      <c r="B297" s="84" t="s">
+    <row r="297" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A297" s="86"/>
+      <c r="B297" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="C297" s="80">
+      <c r="C297" s="49">
         <v>251978.57177243874</v>
       </c>
-      <c r="D297" s="81">
+      <c r="D297" s="21">
         <v>444885.52470570581</v>
       </c>
-      <c r="E297" s="81">
+      <c r="E297" s="21">
         <v>177015.91697160891</v>
       </c>
-      <c r="F297" s="81">
+      <c r="F297" s="21">
         <v>36549.671021279159</v>
       </c>
-      <c r="G297" s="81">
+      <c r="G297" s="21">
         <v>162941.12280194095</v>
       </c>
-      <c r="H297" s="81">
+      <c r="H297" s="21">
         <v>271746.7448521434</v>
       </c>
-      <c r="I297" s="81">
+      <c r="I297" s="21">
         <v>165093.82100197411</v>
       </c>
-      <c r="J297" s="81">
+      <c r="J297" s="21">
         <v>135291.04542362181</v>
       </c>
-      <c r="K297" s="81">
+      <c r="K297" s="21">
         <v>137109.43372061962</v>
       </c>
-      <c r="L297" s="82">
+      <c r="L297" s="22">
         <v>225536.5068935263</v>
       </c>
-      <c r="M297" s="80">
+      <c r="M297" s="49">
         <v>164.87226453514404</v>
       </c>
-      <c r="N297" s="81">
+      <c r="N297" s="21">
         <v>173.4971116169072</v>
       </c>
-      <c r="O297" s="81">
+      <c r="O297" s="21">
         <v>88.00599169849977</v>
       </c>
-      <c r="P297" s="81">
+      <c r="P297" s="21">
         <v>103.07220676213686</v>
       </c>
-      <c r="Q297" s="81">
+      <c r="Q297" s="21">
         <v>94.242241214447574</v>
       </c>
-      <c r="R297" s="81">
+      <c r="R297" s="21">
         <v>286.66733710676772</v>
       </c>
-      <c r="S297" s="81">
+      <c r="S297" s="21">
         <v>112.99603698848317</v>
       </c>
-      <c r="T297" s="81">
+      <c r="T297" s="21">
         <v>120.29812019497344</v>
       </c>
-      <c r="U297" s="81">
+      <c r="U297" s="21">
         <v>231.4323227479116</v>
       </c>
-      <c r="V297" s="82">
+      <c r="V297" s="22">
         <v>81.259197969232545</v>
       </c>
     </row>
     <row r="298" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A298" s="13" t="s">
+      <c r="A298" s="86"/>
+      <c r="B298" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C298" s="49">
+        <v>248392.67364460917</v>
+      </c>
+      <c r="D298" s="21">
+        <v>427224.52960904449</v>
+      </c>
+      <c r="E298" s="21">
+        <v>187473.96270428976</v>
+      </c>
+      <c r="F298" s="21">
+        <v>40506.510377313818</v>
+      </c>
+      <c r="G298" s="21">
+        <v>81136.921025048301</v>
+      </c>
+      <c r="H298" s="21">
+        <v>345861.29827497929</v>
+      </c>
+      <c r="I298" s="21">
+        <v>217220.53818710631</v>
+      </c>
+      <c r="J298" s="21">
+        <v>124786.5775587254</v>
+      </c>
+      <c r="K298" s="21">
+        <v>92041.155543284345</v>
+      </c>
+      <c r="L298" s="22">
+        <v>442028.33973298414</v>
+      </c>
+      <c r="M298" s="49">
+        <v>183.71577508366977</v>
+      </c>
+      <c r="N298" s="21">
+        <v>177.06409019490036</v>
+      </c>
+      <c r="O298" s="21">
+        <v>87.762800862710947</v>
+      </c>
+      <c r="P298" s="21">
+        <v>113.22887047147169</v>
+      </c>
+      <c r="Q298" s="21">
+        <v>65.634370947794736</v>
+      </c>
+      <c r="R298" s="21">
+        <v>364.93519151613356</v>
+      </c>
+      <c r="S298" s="21">
+        <v>139.70046540564346</v>
+      </c>
+      <c r="T298" s="21">
+        <v>104.92662326651076</v>
+      </c>
+      <c r="U298" s="21">
+        <v>351.30406573668495</v>
+      </c>
+      <c r="V298" s="22">
+        <v>142.03151496560002</v>
+      </c>
+    </row>
+    <row r="299" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A299" s="86"/>
+      <c r="B299" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C299" s="49">
+        <v>224331.56039007733</v>
+      </c>
+      <c r="D299" s="21">
+        <v>420594.12579601962</v>
+      </c>
+      <c r="E299" s="21">
+        <v>163072.10596705927</v>
+      </c>
+      <c r="F299" s="21">
+        <v>43799.248043499269</v>
+      </c>
+      <c r="G299" s="21">
+        <v>85711.985965710293</v>
+      </c>
+      <c r="H299" s="21">
+        <v>267128.06331770989</v>
+      </c>
+      <c r="I299" s="21">
+        <v>169252.70316895412</v>
+      </c>
+      <c r="J299" s="21">
+        <v>101861.25982099187</v>
+      </c>
+      <c r="K299" s="21">
+        <v>95198.00497763796</v>
+      </c>
+      <c r="L299" s="22">
+        <v>390587.3787477861</v>
+      </c>
+      <c r="M299" s="49">
+        <v>142.52225330533943</v>
+      </c>
+      <c r="N299" s="21">
+        <v>179.25132305203141</v>
+      </c>
+      <c r="O299" s="21">
+        <v>75.8267469754784</v>
+      </c>
+      <c r="P299" s="21">
+        <v>120.65254295809585</v>
+      </c>
+      <c r="Q299" s="21">
+        <v>49.015043935196324</v>
+      </c>
+      <c r="R299" s="21">
+        <v>274.94528071221379</v>
+      </c>
+      <c r="S299" s="21">
+        <v>104.02872073021872</v>
+      </c>
+      <c r="T299" s="21">
+        <v>81.526655937193027</v>
+      </c>
+      <c r="U299" s="21">
+        <v>170.63957769177935</v>
+      </c>
+      <c r="V299" s="22">
+        <v>144.28732022960577</v>
+      </c>
+    </row>
+    <row r="300" spans="1:22" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A300" s="100"/>
+      <c r="B300" s="84" t="s">
+        <v>21</v>
+      </c>
+      <c r="C300" s="80">
+        <v>261020.26204074433</v>
+      </c>
+      <c r="D300" s="81">
+        <v>453597.3463528193</v>
+      </c>
+      <c r="E300" s="81">
+        <v>115611.0525401566</v>
+      </c>
+      <c r="F300" s="81">
+        <v>30024.584521064004</v>
+      </c>
+      <c r="G300" s="81">
+        <v>93477.584523507539</v>
+      </c>
+      <c r="H300" s="81">
+        <v>356494.62066558329</v>
+      </c>
+      <c r="I300" s="81">
+        <v>242025.38420826456</v>
+      </c>
+      <c r="J300" s="81">
+        <v>134462.86187378434</v>
+      </c>
+      <c r="K300" s="81">
+        <v>108241.87112889507</v>
+      </c>
+      <c r="L300" s="82">
+        <v>433228.0990092482</v>
+      </c>
+      <c r="M300" s="80">
+        <v>155.04950424280682</v>
+      </c>
+      <c r="N300" s="81">
+        <v>190.0157361790352</v>
+      </c>
+      <c r="O300" s="81">
+        <v>53.873271920157777</v>
+      </c>
+      <c r="P300" s="81">
+        <v>81.704420582298638</v>
+      </c>
+      <c r="Q300" s="81">
+        <v>43.54964282970883</v>
+      </c>
+      <c r="R300" s="81">
+        <v>355.86186970652363</v>
+      </c>
+      <c r="S300" s="81">
+        <v>146.64798317586622</v>
+      </c>
+      <c r="T300" s="81">
+        <v>98.421741649143613</v>
+      </c>
+      <c r="U300" s="81">
+        <v>166.16593004890765</v>
+      </c>
+      <c r="V300" s="82">
+        <v>155.34373303885872</v>
+      </c>
+    </row>
+    <row r="301" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A301" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C298" s="2"/>
-      <c r="D298" s="1"/>
-      <c r="E298" s="1"/>
-      <c r="F298" s="1"/>
-      <c r="G298" s="1"/>
-      <c r="H298" s="2"/>
-      <c r="I298" s="2"/>
-      <c r="J298" s="2"/>
-      <c r="K298" s="2"/>
-      <c r="L298" s="2"/>
-      <c r="M298" s="83"/>
-      <c r="N298" s="45"/>
-      <c r="O298" s="45"/>
-      <c r="P298" s="45"/>
-      <c r="Q298" s="45"/>
-      <c r="R298" s="45"/>
-      <c r="S298" s="45"/>
-      <c r="T298" s="45"/>
-      <c r="U298" s="45"/>
-      <c r="V298" s="45"/>
-    </row>
-    <row r="299" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A299" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C299" s="2"/>
-      <c r="D299" s="1"/>
-      <c r="E299" s="1"/>
-      <c r="F299" s="1"/>
-      <c r="G299" s="1"/>
-      <c r="H299" s="2"/>
-      <c r="I299" s="2"/>
-      <c r="J299" s="2"/>
-      <c r="K299" s="2"/>
-      <c r="L299" s="2"/>
-      <c r="M299" s="2"/>
-      <c r="N299" s="2"/>
-      <c r="O299" s="1"/>
-      <c r="P299" s="1"/>
-      <c r="Q299" s="1"/>
-      <c r="R299" s="1"/>
-      <c r="S299" s="2"/>
-      <c r="T299" s="2"/>
-      <c r="U299" s="2"/>
-      <c r="V299" s="2"/>
-    </row>
-    <row r="300" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="C300" s="2"/>
-      <c r="D300" s="1"/>
-      <c r="E300" s="1"/>
-      <c r="F300" s="1"/>
-      <c r="G300" s="1"/>
-      <c r="H300" s="2"/>
-      <c r="I300" s="2"/>
-      <c r="J300" s="2"/>
-      <c r="K300" s="2"/>
-      <c r="L300" s="2"/>
-      <c r="M300" s="2"/>
-      <c r="N300" s="2"/>
-      <c r="O300" s="1"/>
-      <c r="P300" s="1"/>
-      <c r="Q300" s="1"/>
-      <c r="R300" s="1"/>
-      <c r="S300" s="2"/>
-      <c r="T300" s="2"/>
-      <c r="U300" s="2"/>
-      <c r="V300" s="2"/>
-    </row>
-    <row r="301" spans="1:22" x14ac:dyDescent="0.2">
       <c r="C301" s="2"/>
       <c r="D301" s="1"/>
       <c r="E301" s="1"/>
@@ -21537,18 +21677,21 @@
       <c r="J301" s="2"/>
       <c r="K301" s="2"/>
       <c r="L301" s="2"/>
-      <c r="M301" s="2"/>
-      <c r="N301" s="2"/>
-      <c r="O301" s="1"/>
-      <c r="P301" s="1"/>
-      <c r="Q301" s="1"/>
-      <c r="R301" s="1"/>
-      <c r="S301" s="2"/>
-      <c r="T301" s="2"/>
-      <c r="U301" s="2"/>
-      <c r="V301" s="2"/>
+      <c r="M301" s="83"/>
+      <c r="N301" s="45"/>
+      <c r="O301" s="45"/>
+      <c r="P301" s="45"/>
+      <c r="Q301" s="45"/>
+      <c r="R301" s="45"/>
+      <c r="S301" s="45"/>
+      <c r="T301" s="45"/>
+      <c r="U301" s="45"/>
+      <c r="V301" s="45"/>
     </row>
     <row r="302" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A302" s="14" t="s">
+        <v>58</v>
+      </c>
       <c r="C302" s="2"/>
       <c r="D302" s="1"/>
       <c r="E302" s="1"/>
@@ -21813,34 +21956,70 @@
       <c r="V313" s="2"/>
     </row>
     <row r="314" spans="3:22" x14ac:dyDescent="0.2">
-      <c r="D314" s="8"/>
-      <c r="E314" s="8"/>
-      <c r="F314" s="8"/>
-      <c r="G314" s="8"/>
-      <c r="O314" s="3"/>
-      <c r="P314" s="3"/>
-      <c r="Q314" s="3"/>
-      <c r="R314" s="3"/>
+      <c r="C314" s="2"/>
+      <c r="D314" s="1"/>
+      <c r="E314" s="1"/>
+      <c r="F314" s="1"/>
+      <c r="G314" s="1"/>
+      <c r="H314" s="2"/>
+      <c r="I314" s="2"/>
+      <c r="J314" s="2"/>
+      <c r="K314" s="2"/>
+      <c r="L314" s="2"/>
+      <c r="M314" s="2"/>
+      <c r="N314" s="2"/>
+      <c r="O314" s="1"/>
+      <c r="P314" s="1"/>
+      <c r="Q314" s="1"/>
+      <c r="R314" s="1"/>
+      <c r="S314" s="2"/>
+      <c r="T314" s="2"/>
+      <c r="U314" s="2"/>
+      <c r="V314" s="2"/>
     </row>
     <row r="315" spans="3:22" x14ac:dyDescent="0.2">
-      <c r="D315" s="8"/>
-      <c r="E315" s="8"/>
-      <c r="F315" s="8"/>
-      <c r="G315" s="8"/>
-      <c r="O315" s="3"/>
-      <c r="P315" s="3"/>
-      <c r="Q315" s="3"/>
-      <c r="R315" s="3"/>
+      <c r="C315" s="2"/>
+      <c r="D315" s="1"/>
+      <c r="E315" s="1"/>
+      <c r="F315" s="1"/>
+      <c r="G315" s="1"/>
+      <c r="H315" s="2"/>
+      <c r="I315" s="2"/>
+      <c r="J315" s="2"/>
+      <c r="K315" s="2"/>
+      <c r="L315" s="2"/>
+      <c r="M315" s="2"/>
+      <c r="N315" s="2"/>
+      <c r="O315" s="1"/>
+      <c r="P315" s="1"/>
+      <c r="Q315" s="1"/>
+      <c r="R315" s="1"/>
+      <c r="S315" s="2"/>
+      <c r="T315" s="2"/>
+      <c r="U315" s="2"/>
+      <c r="V315" s="2"/>
     </row>
     <row r="316" spans="3:22" x14ac:dyDescent="0.2">
-      <c r="D316" s="8"/>
-      <c r="E316" s="8"/>
-      <c r="F316" s="8"/>
-      <c r="G316" s="8"/>
-      <c r="O316" s="3"/>
-      <c r="P316" s="3"/>
-      <c r="Q316" s="3"/>
-      <c r="R316" s="3"/>
+      <c r="C316" s="2"/>
+      <c r="D316" s="1"/>
+      <c r="E316" s="1"/>
+      <c r="F316" s="1"/>
+      <c r="G316" s="1"/>
+      <c r="H316" s="2"/>
+      <c r="I316" s="2"/>
+      <c r="J316" s="2"/>
+      <c r="K316" s="2"/>
+      <c r="L316" s="2"/>
+      <c r="M316" s="2"/>
+      <c r="N316" s="2"/>
+      <c r="O316" s="1"/>
+      <c r="P316" s="1"/>
+      <c r="Q316" s="1"/>
+      <c r="R316" s="1"/>
+      <c r="S316" s="2"/>
+      <c r="T316" s="2"/>
+      <c r="U316" s="2"/>
+      <c r="V316" s="2"/>
     </row>
     <row r="317" spans="3:22" x14ac:dyDescent="0.2">
       <c r="D317" s="8"/>
@@ -23432,19 +23611,39 @@
       <c r="Q475" s="3"/>
       <c r="R475" s="3"/>
     </row>
+    <row r="476" spans="4:18" x14ac:dyDescent="0.2">
+      <c r="D476" s="8"/>
+      <c r="E476" s="8"/>
+      <c r="F476" s="8"/>
+      <c r="G476" s="8"/>
+      <c r="O476" s="3"/>
+      <c r="P476" s="3"/>
+      <c r="Q476" s="3"/>
+      <c r="R476" s="3"/>
+    </row>
+    <row r="477" spans="4:18" x14ac:dyDescent="0.2">
+      <c r="D477" s="8"/>
+      <c r="E477" s="8"/>
+      <c r="F477" s="8"/>
+      <c r="G477" s="8"/>
+      <c r="O477" s="3"/>
+      <c r="P477" s="3"/>
+      <c r="Q477" s="3"/>
+      <c r="R477" s="3"/>
+    </row>
+    <row r="478" spans="4:18" x14ac:dyDescent="0.2">
+      <c r="D478" s="8"/>
+      <c r="E478" s="8"/>
+      <c r="F478" s="8"/>
+      <c r="G478" s="8"/>
+      <c r="O478" s="3"/>
+      <c r="P478" s="3"/>
+      <c r="Q478" s="3"/>
+      <c r="R478" s="3"/>
+    </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A235:A246"/>
-    <mergeCell ref="A163:A174"/>
-    <mergeCell ref="A151:A162"/>
-    <mergeCell ref="M2:V2"/>
-    <mergeCell ref="A7:A18"/>
-    <mergeCell ref="A19:A30"/>
-    <mergeCell ref="A31:A42"/>
-    <mergeCell ref="A43:A54"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="A295:A297"/>
+    <mergeCell ref="A295:A300"/>
     <mergeCell ref="A283:A294"/>
     <mergeCell ref="A103:A114"/>
     <mergeCell ref="A115:A126"/>
@@ -23460,6 +23659,16 @@
     <mergeCell ref="A139:A150"/>
     <mergeCell ref="A259:A270"/>
     <mergeCell ref="A247:A258"/>
+    <mergeCell ref="A235:A246"/>
+    <mergeCell ref="A163:A174"/>
+    <mergeCell ref="A151:A162"/>
+    <mergeCell ref="M2:V2"/>
+    <mergeCell ref="A7:A18"/>
+    <mergeCell ref="A19:A30"/>
+    <mergeCell ref="A31:A42"/>
+    <mergeCell ref="A43:A54"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
@@ -23596,7 +23805,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="59" t="s">
         <v>40</v>
       </c>
@@ -23604,7 +23813,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="59" t="s">
         <v>41</v>
       </c>
@@ -23620,7 +23829,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="69" t="s">
         <v>44</v>
       </c>

</xml_diff>